<commit_message>
Remove founder stipend from the PROTOPUS ask: ₹19 lakh
Set the founder stipend to zero in the PoC Budget sheet. The ask rounds to
₹19,00,000 with a ₹1,01,735 reserve (7.5% of non-hardware lines); the
too-early comparison becomes ₹29 lakh. Deck slides 11-14 updated to match.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015VN4M2s8EYDB3tD3YjqASb
</commit_message>
<xml_diff>
--- a/PROTOPUS/PROTOPUS_Baker_Mixer_BOM_and_Costing.xlsx
+++ b/PROTOPUS/PROTOPUS_Baker_Mixer_BOM_and_Costing.xlsx
@@ -149,7 +149,7 @@
     <t xml:space="preserve">Founder stipend per month</t>
   </si>
   <si>
-    <t xml:space="preserve">ASSUMPTION: modest living stipend; set to 0 if the funder does not allow it</t>
+    <t xml:space="preserve">Deducted: the founder takes no stipend during the proof of concept</t>
   </si>
   <si>
     <t xml:space="preserve">Proto software + compute per month</t>
@@ -2201,11 +2201,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="33627937"/>
-        <c:axId val="25503896"/>
+        <c:axId val="19349946"/>
+        <c:axId val="25974372"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="33627937"/>
+        <c:axId val="19349946"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2237,7 +2237,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="25503896"/>
+        <c:crossAx val="25974372"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2245,7 +2245,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="25503896"/>
+        <c:axId val="25974372"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2287,7 +2287,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="33627937"/>
+        <c:crossAx val="19349946"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2515,11 +2515,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="53678661"/>
-        <c:axId val="20665165"/>
+        <c:axId val="80062474"/>
+        <c:axId val="71721433"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="53678661"/>
+        <c:axId val="80062474"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -2551,7 +2551,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="20665165"/>
+        <c:crossAx val="71721433"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2559,7 +2559,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="20665165"/>
+        <c:axId val="71721433"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2591,7 +2591,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="53678661"/>
+        <c:crossAx val="80062474"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2759,11 +2759,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="30302956"/>
-        <c:axId val="30836831"/>
+        <c:axId val="71780562"/>
+        <c:axId val="90186796"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="30302956"/>
+        <c:axId val="71780562"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -2795,7 +2795,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="30836831"/>
+        <c:crossAx val="90186796"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2803,7 +2803,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="30836831"/>
+        <c:axId val="90186796"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2835,7 +2835,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="30302956"/>
+        <c:crossAx val="71780562"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4109,7 +4109,7 @@
         <v>36</v>
       </c>
       <c r="B9" s="19" t="n">
-        <v>20000</v>
+        <v>0</v>
       </c>
       <c r="C9" s="18" t="s">
         <v>37</v>
@@ -4270,7 +4270,7 @@
       </c>
       <c r="B21" s="7" t="n">
         <f aca="false">$B$9*$B$6</f>
-        <v>180000</v>
+        <v>0</v>
       </c>
       <c r="C21" s="16" t="s">
         <v>63</v>
@@ -4374,7 +4374,7 @@
       </c>
       <c r="B27" s="23" t="n">
         <f aca="false">SUM(B15:B26)</f>
-        <v>1978264.8756</v>
+        <v>1798264.8756</v>
       </c>
       <c r="C27" s="24"/>
       <c r="D27" s="24"/>
@@ -4385,7 +4385,7 @@
       </c>
       <c r="B28" s="25" t="n">
         <f aca="false">SUMIF(E15:E26,"N",B15:B26)</f>
-        <v>1530000</v>
+        <v>1350000</v>
       </c>
       <c r="C28" s="24"/>
       <c r="D28" s="24"/>
@@ -4396,7 +4396,7 @@
       </c>
       <c r="B29" s="27" t="n">
         <f aca="false">ROUND((B27+B28*$B$11)/100000,0)*100000</f>
-        <v>2100000</v>
+        <v>1900000</v>
       </c>
       <c r="C29" s="28"/>
       <c r="D29" s="28"/>
@@ -4407,11 +4407,11 @@
       </c>
       <c r="B30" s="25" t="n">
         <f aca="false">B29-B27</f>
-        <v>121735.1244</v>
+        <v>101735.1244</v>
       </c>
       <c r="C30" s="29" t="n">
         <f aca="false">IF(B28=0,0,B30/B28)</f>
-        <v>0.0795654407843138</v>
+        <v>0.0753593514074075</v>
       </c>
       <c r="D30" s="18" t="s">
         <v>84</v>
@@ -4443,7 +4443,7 @@
       </c>
       <c r="C34" s="30" t="n">
         <f aca="false">IF($B$29=0,0,B34/$B$29)</f>
-        <v>0.213459464571429</v>
+        <v>0.235928881894737</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4456,7 +4456,7 @@
       </c>
       <c r="C35" s="30" t="n">
         <f aca="false">IF($B$29=0,0,B35/$B$29)</f>
-        <v>0.104761904761905</v>
+        <v>0.115789473684211</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4465,11 +4465,11 @@
       </c>
       <c r="B36" s="7" t="n">
         <f aca="false">SUMIF($C$15:$C$26,A36,$B$15:$B$26)</f>
-        <v>900000</v>
+        <v>720000</v>
       </c>
       <c r="C36" s="30" t="n">
         <f aca="false">IF($B$29=0,0,B36/$B$29)</f>
-        <v>0.428571428571429</v>
+        <v>0.378947368421053</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4482,7 +4482,7 @@
       </c>
       <c r="C37" s="30" t="n">
         <f aca="false">IF($B$29=0,0,B37/$B$29)</f>
-        <v>0.0642857142857143</v>
+        <v>0.0710526315789474</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4495,7 +4495,7 @@
       </c>
       <c r="C38" s="30" t="n">
         <f aca="false">IF($B$29=0,0,B38/$B$29)</f>
-        <v>0.0714285714285714</v>
+        <v>0.0789473684210526</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4504,11 +4504,11 @@
       </c>
       <c r="B39" s="7" t="n">
         <f aca="false">SUMIF($C$15:$C$26,A39,$B$15:$B$26)+B30</f>
-        <v>246735.1244</v>
+        <v>226735.1244</v>
       </c>
       <c r="C39" s="30" t="n">
         <f aca="false">IF($B$29=0,0,B39/$B$29)</f>
-        <v>0.117492916380952</v>
+        <v>0.119334276</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4559,7 +4559,7 @@
       </c>
       <c r="B45" s="34" t="n">
         <f aca="false">B29</f>
-        <v>2100000</v>
+        <v>1900000</v>
       </c>
       <c r="C45" s="28" t="str">
         <f aca="false">B6&amp;" months"</f>
@@ -4575,7 +4575,7 @@
       </c>
       <c r="B46" s="7" t="n">
         <f aca="false">ROUND((B29+'Baker Final Cost'!B10+$B$8*$B$6+250000)/100000,0)*100000</f>
-        <v>3100000</v>
+        <v>2900000</v>
       </c>
       <c r="C46" s="24" t="str">
         <f aca="false">B6&amp;" months"</f>

</xml_diff>

<commit_message>
Size the PROTOPUS team to one software + firmware engineer: ₹16 lakh ask
One engineer covering software and firmware at ₹50,000/month replaces two
engineers; the founder covers mechanical and electronics. The ask rounds to
₹16,00,000 with a ₹71,735 reserve; the too-early option becomes ₹27 lakh.
Deck slides 11-15 and the thank-you slide's hiring line updated to match.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015VN4M2s8EYDB3tD3YjqASb
</commit_message>
<xml_diff>
--- a/PROTOPUS/PROTOPUS_Baker_Mixer_BOM_and_Costing.xlsx
+++ b/PROTOPUS/PROTOPUS_Baker_Mixer_BOM_and_Costing.xlsx
@@ -134,16 +134,16 @@
     <t xml:space="preserve">6 months to proof of concept (deck timeline) + 3 months to close the next round</t>
   </si>
   <si>
-    <t xml:space="preserve">Engineers (firmware + mechanical)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Deck: hiring next, a firmware engineer and a mechanical engineer</t>
+    <t xml:space="preserve">Engineers (software + firmware)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One software engineer who also writes the firmware; the founder covers mechanical and electronics</t>
   </si>
   <si>
     <t xml:space="preserve">Cost per engineer per month</t>
   </si>
   <si>
-    <t xml:space="preserve">ASSUMPTION: entry-level embedded/mechanical engineer in Delhi; the ₹10L ask assumed ₹25,000</t>
+    <t xml:space="preserve">ASSUMPTION: software + firmware in one person, Delhi; ₹40,000 would lower the ask to ₹15L. The ₹10L ask assumed ₹25,000</t>
   </si>
   <si>
     <t xml:space="preserve">Founder stipend per month</t>
@@ -335,10 +335,10 @@
     <t xml:space="preserve">Too early</t>
   </si>
   <si>
-    <t xml:space="preserve">Adds a second Baker for a studio, a third engineer and China samples + trip. That is seed-round work: it spends money before the PoC has removed the risk.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Too-early option adds: second Baker at prototype cost, one more engineer for the runway, ₹2,50,000 for China DFM samples + one Shenzhen trip (ASSUMPTION).</t>
+    <t xml:space="preserve">Adds a second Baker for a studio, a mechanical engineer and China samples + trip. That is seed-round work: it spends money before the PoC has removed the risk.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Too-early option adds: second Baker at prototype cost, one more engineer (mechanical) for the runway, ₹2,50,000 for China DFM samples + one Shenzhen trip (ASSUMPTION).</t>
   </si>
   <si>
     <t xml:space="preserve">Baker — prototype bill of materials (India-sourced)</t>
@@ -2201,11 +2201,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="19349946"/>
-        <c:axId val="25974372"/>
+        <c:axId val="95840242"/>
+        <c:axId val="31076756"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="19349946"/>
+        <c:axId val="95840242"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2237,7 +2237,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="25974372"/>
+        <c:crossAx val="31076756"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2245,7 +2245,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="25974372"/>
+        <c:axId val="31076756"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2287,7 +2287,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="19349946"/>
+        <c:crossAx val="95840242"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2515,11 +2515,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="80062474"/>
-        <c:axId val="71721433"/>
+        <c:axId val="69033556"/>
+        <c:axId val="49193885"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="80062474"/>
+        <c:axId val="69033556"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -2551,7 +2551,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="71721433"/>
+        <c:crossAx val="49193885"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2559,7 +2559,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="71721433"/>
+        <c:axId val="49193885"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2591,7 +2591,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="80062474"/>
+        <c:crossAx val="69033556"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2759,11 +2759,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="71780562"/>
-        <c:axId val="90186796"/>
+        <c:axId val="47919889"/>
+        <c:axId val="23178642"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="71780562"/>
+        <c:axId val="47919889"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -2795,7 +2795,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="90186796"/>
+        <c:crossAx val="23178642"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2803,7 +2803,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="90186796"/>
+        <c:axId val="23178642"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2835,7 +2835,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="71780562"/>
+        <c:crossAx val="47919889"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4087,7 +4087,7 @@
         <v>32</v>
       </c>
       <c r="B7" s="17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C7" s="18" t="s">
         <v>33</v>
@@ -4098,7 +4098,7 @@
         <v>34</v>
       </c>
       <c r="B8" s="19" t="n">
-        <v>40000</v>
+        <v>50000</v>
       </c>
       <c r="C8" s="18" t="s">
         <v>35</v>
@@ -4252,7 +4252,7 @@
       </c>
       <c r="B20" s="7" t="n">
         <f aca="false">$B$7*$B$8*$B$6</f>
-        <v>720000</v>
+        <v>450000</v>
       </c>
       <c r="C20" s="16" t="s">
         <v>63</v>
@@ -4374,7 +4374,7 @@
       </c>
       <c r="B27" s="23" t="n">
         <f aca="false">SUM(B15:B26)</f>
-        <v>1798264.8756</v>
+        <v>1528264.8756</v>
       </c>
       <c r="C27" s="24"/>
       <c r="D27" s="24"/>
@@ -4385,7 +4385,7 @@
       </c>
       <c r="B28" s="25" t="n">
         <f aca="false">SUMIF(E15:E26,"N",B15:B26)</f>
-        <v>1350000</v>
+        <v>1080000</v>
       </c>
       <c r="C28" s="24"/>
       <c r="D28" s="24"/>
@@ -4396,7 +4396,7 @@
       </c>
       <c r="B29" s="27" t="n">
         <f aca="false">ROUND((B27+B28*$B$11)/100000,0)*100000</f>
-        <v>1900000</v>
+        <v>1600000</v>
       </c>
       <c r="C29" s="28"/>
       <c r="D29" s="28"/>
@@ -4407,11 +4407,11 @@
       </c>
       <c r="B30" s="25" t="n">
         <f aca="false">B29-B27</f>
-        <v>101735.1244</v>
+        <v>71735.1244000001</v>
       </c>
       <c r="C30" s="29" t="n">
         <f aca="false">IF(B28=0,0,B30/B28)</f>
-        <v>0.0753593514074075</v>
+        <v>0.0664214114814816</v>
       </c>
       <c r="D30" s="18" t="s">
         <v>84</v>
@@ -4443,7 +4443,7 @@
       </c>
       <c r="C34" s="30" t="n">
         <f aca="false">IF($B$29=0,0,B34/$B$29)</f>
-        <v>0.235928881894737</v>
+        <v>0.28016554725</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4456,7 +4456,7 @@
       </c>
       <c r="C35" s="30" t="n">
         <f aca="false">IF($B$29=0,0,B35/$B$29)</f>
-        <v>0.115789473684211</v>
+        <v>0.1375</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4465,11 +4465,11 @@
       </c>
       <c r="B36" s="7" t="n">
         <f aca="false">SUMIF($C$15:$C$26,A36,$B$15:$B$26)</f>
-        <v>720000</v>
+        <v>450000</v>
       </c>
       <c r="C36" s="30" t="n">
         <f aca="false">IF($B$29=0,0,B36/$B$29)</f>
-        <v>0.378947368421053</v>
+        <v>0.28125</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4482,7 +4482,7 @@
       </c>
       <c r="C37" s="30" t="n">
         <f aca="false">IF($B$29=0,0,B37/$B$29)</f>
-        <v>0.0710526315789474</v>
+        <v>0.084375</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4495,7 +4495,7 @@
       </c>
       <c r="C38" s="30" t="n">
         <f aca="false">IF($B$29=0,0,B38/$B$29)</f>
-        <v>0.0789473684210526</v>
+        <v>0.09375</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4504,11 +4504,11 @@
       </c>
       <c r="B39" s="7" t="n">
         <f aca="false">SUMIF($C$15:$C$26,A39,$B$15:$B$26)+B30</f>
-        <v>226735.1244</v>
+        <v>196735.1244</v>
       </c>
       <c r="C39" s="30" t="n">
         <f aca="false">IF($B$29=0,0,B39/$B$29)</f>
-        <v>0.119334276</v>
+        <v>0.12295945275</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4559,7 +4559,7 @@
       </c>
       <c r="B45" s="34" t="n">
         <f aca="false">B29</f>
-        <v>1900000</v>
+        <v>1600000</v>
       </c>
       <c r="C45" s="28" t="str">
         <f aca="false">B6&amp;" months"</f>
@@ -4575,7 +4575,7 @@
       </c>
       <c r="B46" s="7" t="n">
         <f aca="false">ROUND((B29+'Baker Final Cost'!B10+$B$8*$B$6+250000)/100000,0)*100000</f>
-        <v>2900000</v>
+        <v>2700000</v>
       </c>
       <c r="C46" s="24" t="str">
         <f aca="false">B6&amp;" months"</f>

</xml_diff>